<commit_message>
Samples Excel file updated for one collection Samples
</commit_message>
<xml_diff>
--- a/inventory-users/datasets/samples.xlsx
+++ b/inventory-users/datasets/samples.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bambund.sharepoint.com/sites/BAMDataStoreRollout-TP5-SchulungundBeratung2/Freigegebene Dokumente/TP5 - Schulung und Beratung/Training_Materials-DataStore/Tutorials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aschelle\workspace\openBIS-data-store-tutorials\inventory-users\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{307B27E4-DAC0-46E2-A87C-BA3F31A2FD5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BBC1222-73F9-444C-8655-1D88742D6097}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B26DA9-8845-4005-BB58-390F6F44069E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="58470" yWindow="405" windowWidth="27300" windowHeight="13650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet0" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="34">
   <si>
     <t>SAMPLE</t>
   </si>
@@ -138,9 +138,6 @@
   </si>
   <si>
     <t>X.1_MATERIALS</t>
-  </si>
-  <si>
-    <t>/X.1_MATERIALS/SAMPLES_SYNTHESIS/COLLECTION_TREATED_SAMPLES</t>
   </si>
 </sst>
 </file>
@@ -225,22 +222,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 4" xfId="2" xr:uid="{58103503-31E1-4E35-A1A4-E69990A7C6CD}"/>
     <cellStyle name="Normal 5" xfId="1" xr:uid="{4364CE09-7437-420A-951B-C0CCE0EC5080}"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -256,9 +250,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -296,7 +290,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -402,7 +396,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -553,42 +547,42 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R8"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -596,17 +590,17 @@
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="5" t="s">
         <v>30</v>
       </c>
       <c r="E4" s="3" t="s">
@@ -652,20 +646,19 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="8"/>
       <c r="G5" t="s">
         <v>22</v>
       </c>
@@ -679,20 +672,19 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="8"/>
       <c r="G6" t="s">
         <v>23</v>
       </c>
@@ -706,20 +698,19 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="9" t="s">
+      <c r="B7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="8"/>
       <c r="G7" s="4" t="s">
         <v>24</v>
       </c>
@@ -733,20 +724,19 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="9" t="s">
+      <c r="B8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="8"/>
       <c r="G8" s="4" t="s">
         <v>25</v>
       </c>
@@ -768,25 +758,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d4726ee-3fa4-4b4f-aa7e-39736bf7daf7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100EDAD2D8B65BB004D846F933953797760" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="85fa1bf82fe312ea6d75f8ef6efa93d0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d4726ee-3fa4-4b4f-aa7e-39736bf7daf7" xmlns:ns3="9faaaee3-3651-4473-96fe-bfd7c1b04dfa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d660665890d5dd31abec9ccbe7d3d4a" ns2:_="" ns3:_="">
     <xsd:import namespace="0d4726ee-3fa4-4b4f-aa7e-39736bf7daf7"/>
@@ -1015,7 +986,53 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d4726ee-3fa4-4b4f-aa7e-39736bf7daf7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8281E022-7C87-4BF5-9601-DD2FE4F0CA95}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="0d4726ee-3fa4-4b4f-aa7e-39736bf7daf7"/>
+    <ds:schemaRef ds:uri="9faaaee3-3651-4473-96fe-bfd7c1b04dfa"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B521658-A164-4B31-9B47-2177D928AC0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44E56622-92B0-4544-869B-B1354D6BE44E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -1032,31 +1049,4 @@
     <ds:schemaRef ds:uri="dc51d558-bfba-4c32-92b9-2c84b939da76"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B521658-A164-4B31-9B47-2177D928AC0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8281E022-7C87-4BF5-9601-DD2FE4F0CA95}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="0d4726ee-3fa4-4b4f-aa7e-39736bf7daf7"/>
-    <ds:schemaRef ds:uri="9faaaee3-3651-4473-96fe-bfd7c1b04dfa"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>